<commit_message>
📋 TA Scan 2026-03-07 20:09 UTC — profilo: msl-veneto
</commit_message>
<xml_diff>
--- a/output/msl-veneto/TA_Monitor_2026-03-07.xlsx
+++ b/output/msl-veneto/TA_Monitor_2026-03-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Posizioni" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Posizioni'!$A$1:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Posizioni'!$A$1:$I$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -497,10 +497,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Recreation Aid (Developmental) NF-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>Speech Therapist - Sost. maternità</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Coloplast</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>indeed</t>
@@ -508,19 +512,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Vicenza, VEN, IT</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>parttime</t>
-        </is>
-      </c>
+          <t>Padova, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f440994f6ab79fdf</t>
+          <t>https://it.indeed.com/viewjob?jk=2b9efae5d2c17f69</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -532,10 +532,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CYS Assistant Director NF-03</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>Clinical Specialist (f/m/d)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>W. L. Gore &amp; Associates</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>indeed</t>
@@ -543,19 +547,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Vicenza, VEN, IT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Verona, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=d8eca911c0b068a2</t>
+          <t>https://it.indeed.com/viewjob?jk=e50b3c514abc4a60</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -567,214 +567,246 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ISF Agente Monomandatario</t>
+          <t>Stack Scaling Engineer (Vanadium Redox Flow Battery (VRFB))</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Neopharmed Gentili S.P.A.</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Verona, Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4379360587</t>
+          <t>https://it.indeed.com/viewjob?jk=b52e9b92e15bc01c</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Informatore Scientifico del Farmaco Dermatologia - Trentino/Veneto</t>
+          <t>BMS Engineer (Flow battery systems)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LHH</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Verona, Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4365567852</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=aa4386d15aac7270</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Informatore Scientifico - ISF - Farma | Treviso e Belluno</t>
+          <t>Research Engineer (Vanadium Extraction &amp; Process Development)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hays</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4378965340</t>
+          <t>https://it.indeed.com/viewjob?jk=088702d5106b703b</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Informatore scientifico commerciale | Veneto</t>
+          <t>Project Manager (Supply Chain Management, Engineering)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PharmaNutra</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Padua, Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4381444347</t>
+          <t>https://it.indeed.com/viewjob?jk=6852551f01e826f7</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Informatore Scientifico Dermatologia e Ginecologia (Area di riferimento Verona/Vicenza/Padova/Rovigo)</t>
+          <t>Senior Software Development Engineer (Computer science, Computer Applications, Engineering)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chaberton Professionals</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4379842560</t>
+          <t>https://it.indeed.com/viewjob?jk=d57f7a10f295812f</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Informatore scientifico</t>
+          <t>Senior Research Scientist (Power Electronics in Flow-based Energy Storages)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pharmera</t>
+          <t>Nanyang Technological University</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Rovigo, Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>One', VEN, IT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4374283868</t>
+          <t>https://it.indeed.com/viewjob?jk=6aeaae0709a22944</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IQVIA Italia Infermiere per attività domiciliari</t>
+          <t>R&amp;D Laboratory Technician</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IQVIA SOLUTIONS ITALY SRL</t>
+          <t>Dentsply Sirona</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -784,7 +816,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>VEN, IT</t>
+          <t>Badia Polesine, VEN, IT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -792,61 +824,57 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=66d69efb805d16b3</t>
+          <t>https://it.indeed.com/viewjob?jk=29ec9b50e9f257c3</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Regulatory Affairs Specialist</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Fidia Pharma</t>
-        </is>
-      </c>
+          <t>Recreation Aid (Developmental) NF-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Abano Terme, Veneto, Italy</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Vicenza, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>parttime</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4378178500</t>
+          <t>https://it.indeed.com/viewjob?jk=f440994f6ab79fdf</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sommelier</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ORIENT EXPRESS</t>
-        </is>
-      </c>
+          <t>CYS Assistant Director NF-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>indeed</t>
@@ -854,7 +882,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Venezia, VEN, IT</t>
+          <t>Vicenza, VEN, IT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -866,63 +894,59 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=8fb90dbba2129d77</t>
+          <t>https://it.indeed.com/viewjob?jk=d8eca911c0b068a2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Victim Advocate</t>
+          <t>ISF Agente Monomandatario</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>US 21st Theater Sustainment Command (TSC)</t>
+          <t>Neopharmed Gentili S.P.A.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Vicenza, VEN, IT</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>parttime, fulltime</t>
-        </is>
-      </c>
+          <t>Verona, Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=91b0952116a54399</t>
+          <t>https://www.linkedin.com/jobs/view/4379360587</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Temporary Clinical Monitor</t>
+          <t>Informatore Scientifico del Farmaco Dermatologia - Trentino/Veneto</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jobbit</t>
+          <t>LHH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -932,7 +956,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Padua, Veneto, Italy</t>
+          <t>Verona, Veneto, Italy</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -940,52 +964,367 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4381699462</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4365567852</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marketing Expert</t>
+          <t>Informatore Scientifico - ISF - Farma | Treviso e Belluno</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fidia Farmaceutici Spa</t>
+          <t>Hays</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Abano Terme, VEN, IT</t>
-        </is>
-      </c>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>https://www.linkedin.com/jobs/view/4378965340</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Informatore scientifico commerciale | Veneto</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PharmaNutra</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Padua, Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4381444347</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Informatore Scientifico Dermatologia e Ginecologia (Area di riferimento Verona/Vicenza/Padova/Rovigo)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chaberton Professionals</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4379842560</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Informatore scientifico</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pharmera</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Rovigo, Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4374283868</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>IQVIA Italia Infermiere per attività domiciliari</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IQVIA SOLUTIONS ITALY SRL</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>VEN, IT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=66d69efb805d16b3</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Specialist</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fidia Pharma</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Abano Terme, Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4378178500</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sommelier</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ORIENT EXPRESS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Venezia, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=8fb90dbba2129d77</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Victim Advocate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>US 21st Theater Sustainment Command (TSC)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Vicenza, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>parttime, fulltime</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=91b0952116a54399</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Temporary Clinical Monitor</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Jobbit</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Padua, Veneto, Italy</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4381699462</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Marketing Expert</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fidia Farmaceutici Spa</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Abano Terme, VEN, IT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
           <t>https://it.indeed.com/viewjob?jk=2a6e5c719a1f7ace</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I15"/>
+  <autoFilter ref="A1:I24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>